<commit_message>
Add Tyler Lewis to UC roster and monthly export row mapping
</commit_message>
<xml_diff>
--- a/templates/Monthly UC 2025 new.xlsx
+++ b/templates/Monthly UC 2025 new.xlsx
@@ -2167,7 +2167,11 @@
       </c>
     </row>
     <row r="31" ht="21" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -2179,7 +2183,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -3763,7 +3771,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -3775,7 +3787,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -5354,7 +5370,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -5366,7 +5386,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -6945,7 +6969,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -6957,7 +6985,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -9760,7 +9792,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -9772,7 +9808,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -11351,7 +11391,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -11363,7 +11407,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -12942,7 +12990,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -12954,7 +13006,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -14534,7 +14590,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -14546,7 +14606,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -16125,7 +16189,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -16137,7 +16205,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -17716,7 +17788,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -17728,7 +17804,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -19308,7 +19388,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -19320,7 +19404,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>
@@ -20899,7 +20987,11 @@
       </c>
     </row>
     <row r="31" ht="24.75" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A31" s="15" t="inlineStr"/>
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="B31" s="52" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
@@ -20911,7 +21003,11 @@
       <c r="J31" s="58" t="n"/>
       <c r="K31" s="58" t="n"/>
       <c r="L31" s="59" t="n"/>
-      <c r="M31" s="30" t="inlineStr"/>
+      <c r="M31" s="30" t="inlineStr">
+        <is>
+          <t>Tyler Lewis</t>
+        </is>
+      </c>
       <c r="N31" s="41" t="n"/>
       <c r="O31" s="41" t="n"/>
       <c r="P31" s="41" t="n"/>

</xml_diff>